<commit_message>
Add Senior-Level Analytics: Statistical A/B Testing (Welch t-test & DiD), Cohort Retention & 12M CLV, Apriori Market Basket Affinity, Q4 Budget Optimizer, 9-Sheet Board Pack & 3-Page Power BI App
</commit_message>
<xml_diff>
--- a/deliverables/Baltic_Loyalty_Performance_Report_Board_Pack.xlsx
+++ b/deliverables/Baltic_Loyalty_Performance_Report_Board_Pack.xlsx
@@ -9,9 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Baltic_Board_Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Campaign_PrePost_ROI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Customer_RFM_Segments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_App_Journey_Funnel" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_POS_Data_Quality_Audit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_AB_Testing_Causal_Uplift" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Customer_RFM_Segments" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Cohort_Retention_Matrix" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_CLV_Churn_Risk_Model" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Market_Basket_Affinity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Q4_Budget_Optimizer" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_POS_Data_Quality_Audit" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +36,32 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00003876"/>
+        <bgColor rgb="00003876"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -55,15 +75,33 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,206 +469,221 @@
   </sheetPr>
   <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Country_Code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Active_Stores</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Total_Transactions</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Total_Net_Sales_EUR</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Loyalty_Scan_Share_Pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Loyalty_Revenue_Share_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Avg_Basket_Loyalty_EUR</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Avg_Basket_Guest_EUR</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Basket_Uplift_EUR</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Basket_Uplift_Pct</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Coupon_Redemption_Rate_Pct</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Total_Promo_Discount_EUR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Lithuania</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="3" t="n">
         <v>87</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>317341</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>7959885.7</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>67.92</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="3" t="n">
         <v>78.98</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="3" t="n">
         <v>29.17</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="3" t="n">
         <v>16.44</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="3" t="n">
         <v>12.73</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="3" t="n">
         <v>77.5</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="3" t="n">
         <v>46.53</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="3" t="n">
         <v>354853.52</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Latvia</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>LV</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="3" t="n">
         <v>119665</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>3026783.7</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>68.13</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="3" t="n">
         <v>79.33</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="3" t="n">
         <v>29.45</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="3" t="n">
         <v>16.41</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="3" t="n">
         <v>13.05</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="3" t="n">
         <v>79.5</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="3" t="n">
         <v>46.38</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="3" t="n">
         <v>133433.64</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Estonia</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>EE</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="3" t="n">
         <v>82994</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>2092350.23</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>68.17</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="3" t="n">
         <v>79.23999999999999</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="3" t="n">
         <v>29.3</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="3" t="n">
         <v>16.44</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="3" t="n">
         <v>12.86</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="3" t="n">
         <v>78.2</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="3" t="n">
         <v>46.62</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="3" t="n">
         <v>93516.39999999999</v>
       </c>
     </row>
@@ -647,1134 +700,1160 @@
   </sheetPr>
   <dimension ref="A1:X13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="27" customWidth="1" min="13" max="13"/>
+    <col width="27" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="32" customWidth="1" min="18" max="18"/>
+    <col width="27" customWidth="1" min="19" max="19"/>
+    <col width="32" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="23" customWidth="1" min="24" max="24"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>campaign_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>campaign_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>mechanic_type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>target_category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>nominal_discount_pct</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>planned_budget_eur</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>commercial_classification</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Redemptions</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Avg_Promo_Item_Spend_EUR</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Avg_Halo_Other_Spend_EUR</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Avg_Gross_Basket_EUR</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Avg_Net_Basket_EUR</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Total_Gross_Revenue_EUR</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Total_Discount_Cost_EUR</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Total_Net_Revenue_EUR</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Total_Net_Margin_EUR</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Cannibalization_Rate_Pct</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>Post_Campaign_Pantry_Dip_Pct</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>Cherry_Picker_Share_Pct</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>True_Incremental_Revenue_EUR</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Net_Incremental_Margin_EUR</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Net_Campaign_ROI_Pct</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>Budget_Utilization_Pct</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>Budget_Variance_EUR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>CMP-09</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Baltic Grill &amp; Fresh Meat -20% Weekend</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Category % Discount</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Meat &amp; Poultry</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="3" t="n">
         <v>64000</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Traffic &amp; Basket Driver (High Halo)</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="3" t="n">
         <v>13681</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="3" t="n">
         <v>6.005493019516117</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="3" t="n">
         <v>33.81241722096338</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="3" t="n">
         <v>39.81791024047949</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="3" t="n">
         <v>38.61679701776186</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="3" t="n">
         <v>544748.83</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="3" t="n">
         <v>16432.43</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2" s="3" t="n">
         <v>528316.4</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" s="3" t="n">
         <v>117030.76</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2" s="3" t="n">
         <v>24.5</v>
       </c>
-      <c r="R2" t="n">
+      <c r="R2" s="3" t="n">
         <v>4.2</v>
       </c>
-      <c r="S2" t="n">
+      <c r="S2" s="3" t="n">
         <v>18.5</v>
       </c>
-      <c r="T2" t="n">
+      <c r="T2" s="3" t="n">
         <v>388405.92</v>
       </c>
-      <c r="U2" t="n">
+      <c r="U2" s="3" t="n">
         <v>78727.02</v>
       </c>
-      <c r="V2" t="n">
+      <c r="V2" s="3" t="n">
         <v>479.1</v>
       </c>
-      <c r="W2" t="n">
+      <c r="W2" s="3" t="n">
         <v>25.7</v>
       </c>
-      <c r="X2" t="n">
+      <c r="X2" s="3" t="n">
         <v>47567.57</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>CMP-06</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Fresh Bananas &amp; Berries -25% App Deal</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Category % Discount</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Fruit &amp; Veg</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="3" t="n">
         <v>39000</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Traffic &amp; Basket Driver (High Halo)</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="3" t="n">
         <v>13692</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="3" t="n">
         <v>6.005511977797254</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="3" t="n">
         <v>33.97005477651183</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="3" t="n">
         <v>39.97556675430909</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="3" t="n">
         <v>38.47419149868536</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="3" t="n">
         <v>547345.46</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="3" t="n">
         <v>20556.83</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O3" s="3" t="n">
         <v>526788.63</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" s="3" t="n">
         <v>113542.58</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="Q3" s="3" t="n">
         <v>24.5</v>
       </c>
-      <c r="R3" t="n">
+      <c r="R3" s="3" t="n">
         <v>4.2</v>
       </c>
-      <c r="S3" t="n">
+      <c r="S3" s="3" t="n">
         <v>18.5</v>
       </c>
-      <c r="T3" t="n">
+      <c r="T3" s="3" t="n">
         <v>390257.31</v>
       </c>
-      <c r="U3" t="n">
+      <c r="U3" s="3" t="n">
         <v>75056.21000000001</v>
       </c>
-      <c r="V3" t="n">
+      <c r="V3" s="3" t="n">
         <v>365.1</v>
       </c>
-      <c r="W3" t="n">
+      <c r="W3" s="3" t="n">
         <v>52.7</v>
       </c>
-      <c r="X3" t="n">
+      <c r="X3" s="3" t="n">
         <v>18443.17</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>CMP-01</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Baltic Fresh Bakery -30% App Coupon</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Category % Discount</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Bakery</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>42000</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Traffic &amp; Basket Driver (High Halo)</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="3" t="n">
         <v>13723</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="3" t="n">
         <v>6.000660205494425</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="3" t="n">
         <v>34.10402535888654</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="3" t="n">
         <v>40.10468556438096</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="3" t="n">
         <v>38.30450193106464</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="3" t="n">
         <v>550356.6</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="3" t="n">
         <v>24703.92</v>
       </c>
-      <c r="O4" t="n">
+      <c r="O4" s="3" t="n">
         <v>525652.6800000001</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" s="3" t="n">
         <v>110133.35</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="Q4" s="3" t="n">
         <v>24.5</v>
       </c>
-      <c r="R4" t="n">
+      <c r="R4" s="3" t="n">
         <v>4.2</v>
       </c>
-      <c r="S4" t="n">
+      <c r="S4" s="3" t="n">
         <v>18.5</v>
       </c>
-      <c r="T4" t="n">
+      <c r="T4" s="3" t="n">
         <v>392404.26</v>
       </c>
-      <c r="U4" t="n">
+      <c r="U4" s="3" t="n">
         <v>71435.12</v>
       </c>
-      <c r="V4" t="n">
+      <c r="V4" s="3" t="n">
         <v>289.2</v>
       </c>
-      <c r="W4" t="n">
+      <c r="W4" s="3" t="n">
         <v>58.8</v>
       </c>
-      <c r="X4" t="n">
+      <c r="X4" s="3" t="n">
         <v>17296.08</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>CMP-03</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Private Label Dairy &amp; Cheese -20%</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Category % Discount</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Dairy &amp; Eggs</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="3" t="n">
         <v>54000</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Core Margin Builder</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="3" t="n">
         <v>13701</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="3" t="n">
         <v>8.752998321290416</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="3" t="n">
         <v>28.73338807386322</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="3" t="n">
         <v>37.48638639515364</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="3" t="n">
         <v>35.73577038172396</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="3" t="n">
         <v>513600.98</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="3" t="n">
         <v>23985.19</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5" s="3" t="n">
         <v>489615.79</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="3" t="n">
         <v>101846.68</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q5" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="R5" t="n">
+      <c r="R5" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="S5" t="n">
+      <c r="S5" s="3" t="n">
         <v>18.5</v>
       </c>
-      <c r="T5" t="n">
+      <c r="T5" s="3" t="n">
         <v>338976.65</v>
       </c>
-      <c r="U5" t="n">
+      <c r="U5" s="3" t="n">
         <v>59064.09</v>
       </c>
-      <c r="V5" t="n">
+      <c r="V5" s="3" t="n">
         <v>246.3</v>
       </c>
-      <c r="W5" t="n">
+      <c r="W5" s="3" t="n">
         <v>44.4</v>
       </c>
-      <c r="X5" t="n">
+      <c r="X5" s="3" t="n">
         <v>30014.81</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>CMP-02</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Spend €30 Get €3 Off Weekend Basket</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Basket Threshold (€30+)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Cross-Category</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="3" t="n">
         <v>68000</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Basket Builder (High ROI)</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="3" t="n">
         <v>13981</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="3" t="n">
         <v>10.96655961662256</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="3" t="n">
         <v>39.96066232744439</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="3" t="n">
         <v>50.92722194406695</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="3" t="n">
         <v>47.92722194406695</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" s="3" t="n">
         <v>712013.49</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="3" t="n">
         <v>41943</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" s="3" t="n">
         <v>670070.49</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6" s="3" t="n">
         <v>132499.67</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q6" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="R6" t="n">
+      <c r="R6" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="S6" t="n">
+      <c r="S6" s="3" t="n">
         <v>11.2</v>
       </c>
-      <c r="T6" t="n">
+      <c r="T6" s="3" t="n">
         <v>554658.51</v>
       </c>
-      <c r="U6" t="n">
+      <c r="U6" s="3" t="n">
         <v>93948.33</v>
       </c>
-      <c r="V6" t="n">
+      <c r="V6" s="3" t="n">
         <v>224</v>
       </c>
-      <c r="W6" t="n">
+      <c r="W6" s="3" t="n">
         <v>61.7</v>
       </c>
-      <c r="X6" t="n">
+      <c r="X6" s="3" t="n">
         <v>26057</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>CMP-10</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Organic &amp; BIO Range -25% Green Week</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Category % Discount</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Organic &amp; Health</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="3" t="n">
         <v>31000</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Core Margin Builder</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="3" t="n">
         <v>13944</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="3" t="n">
         <v>8.738279546758463</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="3" t="n">
         <v>28.69549268502582</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="3" t="n">
         <v>37.43377223178428</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="3" t="n">
         <v>35.24921901893288</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="3" t="n">
         <v>521976.52</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" s="3" t="n">
         <v>30461.41</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O7" s="3" t="n">
         <v>491515.11</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P7" s="3" t="n">
         <v>97422.56</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q7" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="R7" t="n">
+      <c r="R7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="S7" t="n">
+      <c r="S7" s="3" t="n">
         <v>18.5</v>
       </c>
-      <c r="T7" t="n">
+      <c r="T7" s="3" t="n">
         <v>344504.5</v>
       </c>
-      <c r="U7" t="n">
+      <c r="U7" s="3" t="n">
         <v>53942.19</v>
       </c>
-      <c r="V7" t="n">
+      <c r="V7" s="3" t="n">
         <v>177.1</v>
       </c>
-      <c r="W7" t="n">
+      <c r="W7" s="3" t="n">
         <v>98.3</v>
       </c>
-      <c r="X7" t="n">
+      <c r="X7" s="3" t="n">
         <v>538.59</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>CMP-07</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Digital Scratch Card €1.50 Instant Reward</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Gamified Scratch Card</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Cross-Category</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="3" t="n">
         <v>45000</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Retention &amp; Frequency Driver</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="3" t="n">
         <v>13629</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="3" t="n">
         <v>6.986485435468486</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="3" t="n">
         <v>29.96080783623156</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="3" t="n">
         <v>36.94729327170005</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="3" t="n">
         <v>34.20031623743488</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" s="3" t="n">
         <v>503554.66</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N8" s="3" t="n">
         <v>37438.55</v>
       </c>
-      <c r="O8" t="n">
+      <c r="O8" s="3" t="n">
         <v>466116.11</v>
       </c>
-      <c r="P8" t="n">
+      <c r="P8" s="3" t="n">
         <v>85932.14</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q8" s="3" t="n">
         <v>15.5</v>
       </c>
-      <c r="R8" t="n">
+      <c r="R8" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="S8" t="n">
+      <c r="S8" s="3" t="n">
         <v>18.5</v>
       </c>
-      <c r="T8" t="n">
+      <c r="T8" s="3" t="n">
         <v>412914.82</v>
       </c>
-      <c r="U8" t="n">
+      <c r="U8" s="3" t="n">
         <v>63725.58</v>
       </c>
-      <c r="V8" t="n">
+      <c r="V8" s="3" t="n">
         <v>170.2</v>
       </c>
-      <c r="W8" t="n">
+      <c r="W8" s="3" t="n">
         <v>83.2</v>
       </c>
-      <c r="X8" t="n">
+      <c r="X8" s="3" t="n">
         <v>7561.45</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>CMP-12</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Inactive 21-Day Win-Back €4 Off €25</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Win-Back Targeted</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Cross-Category</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="3" t="n">
         <v>36000</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Retention &amp; Frequency Driver</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="3" t="n">
         <v>13641</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="3" t="n">
         <v>6.994323729931824</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="3" t="n">
         <v>29.84416465068543</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="3" t="n">
         <v>36.83848838061726</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="3" t="n">
         <v>34.08263030569606</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="3" t="n">
         <v>502513.82</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="3" t="n">
         <v>37592.66</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O9" s="3" t="n">
         <v>464921.16</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9" s="3" t="n">
         <v>85522.61</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q9" s="3" t="n">
         <v>15.5</v>
       </c>
-      <c r="R9" t="n">
+      <c r="R9" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="S9" t="n">
+      <c r="S9" s="3" t="n">
         <v>18.5</v>
       </c>
-      <c r="T9" t="n">
+      <c r="T9" s="3" t="n">
         <v>412061.33</v>
       </c>
-      <c r="U9" t="n">
+      <c r="U9" s="3" t="n">
         <v>63362.37</v>
       </c>
-      <c r="V9" t="n">
+      <c r="V9" s="3" t="n">
         <v>168.5</v>
       </c>
-      <c r="W9" t="n">
+      <c r="W9" s="3" t="n">
         <v>104.4</v>
       </c>
-      <c r="X9" t="n">
+      <c r="X9" s="3" t="n">
         <v>-1592.66</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>CMP-05</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Spend €40 Get €5 Off Family Stock-Up</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Basket Threshold (€40+)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Cross-Category</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="3" t="n">
         <v>12.5</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="3" t="n">
         <v>75000</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Basket Builder (High ROI)</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="3" t="n">
         <v>13735</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="3" t="n">
         <v>10.98793957044048</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" s="3" t="n">
         <v>39.96668074262832</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="3" t="n">
         <v>50.9546203130688</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="3" t="n">
         <v>45.9546203130688</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" s="3" t="n">
         <v>699861.71</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10" s="3" t="n">
         <v>68675</v>
       </c>
-      <c r="O10" t="n">
+      <c r="O10" s="3" t="n">
         <v>631186.71</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P10" s="3" t="n">
         <v>102791.55</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q10" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="R10" t="n">
+      <c r="R10" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="S10" t="n">
+      <c r="S10" s="3" t="n">
         <v>11.2</v>
       </c>
-      <c r="T10" t="n">
+      <c r="T10" s="3" t="n">
         <v>545192.27</v>
       </c>
-      <c r="U10" t="n">
+      <c r="U10" s="3" t="n">
         <v>64897.11</v>
       </c>
-      <c r="V10" t="n">
+      <c r="V10" s="3" t="n">
         <v>94.5</v>
       </c>
-      <c r="W10" t="n">
+      <c r="W10" s="3" t="n">
         <v>91.59999999999999</v>
       </c>
-      <c r="X10" t="n">
+      <c r="X10" s="3" t="n">
         <v>6325</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>CMP-04</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Imported Coffee Beans XXL -35% Promo</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Deep Item Discount</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Beverages &amp; Coffee</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="3" t="n">
         <v>61000</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Margin Destroyer (Cherry-Picked &amp; Stockpiled)</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="3" t="n">
         <v>13379</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="3" t="n">
         <v>16.47683010688392</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="3" t="n">
         <v>3.333436729202482</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="3" t="n">
         <v>19.8102668360864</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="3" t="n">
         <v>14.04341131624187</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="3" t="n">
         <v>265041.56</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" s="3" t="n">
         <v>77154.75999999999</v>
       </c>
-      <c r="O11" t="n">
+      <c r="O11" s="3" t="n">
         <v>187886.8</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P11" s="3" t="n">
         <v>-12219.81</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q11" s="3" t="n">
         <v>62</v>
       </c>
-      <c r="R11" t="n">
+      <c r="R11" s="3" t="n">
         <v>26.5</v>
       </c>
-      <c r="S11" t="n">
+      <c r="S11" s="3" t="n">
         <v>68.40000000000001</v>
       </c>
-      <c r="T11" t="n">
+      <c r="T11" s="3" t="n">
         <v>30479.78</v>
       </c>
-      <c r="U11" t="n">
+      <c r="U11" s="3" t="n">
         <v>-69687.21000000001</v>
       </c>
-      <c r="V11" t="n">
+      <c r="V11" s="3" t="n">
         <v>-90.3</v>
       </c>
-      <c r="W11" t="n">
+      <c r="W11" s="3" t="n">
         <v>126.5</v>
       </c>
-      <c r="X11" t="n">
+      <c r="X11" s="3" t="n">
         <v>-16154.76</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>CMP-11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Household Detergent XXL -40% Coupon</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Deep Item Discount</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Household</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="3" t="n">
         <v>52000</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Margin Destroyer (Cherry-Picked &amp; Stockpiled)</t>
         </is>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="3" t="n">
         <v>13806</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="3" t="n">
         <v>16.49824858757062</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J12" s="3" t="n">
         <v>3.344019991308127</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="3" t="n">
         <v>19.84226857887875</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="3" t="n">
         <v>13.24294509633493</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="3" t="n">
         <v>273942.36</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12" s="3" t="n">
         <v>91110.25999999999</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O12" s="3" t="n">
         <v>182832.1</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P12" s="3" t="n">
         <v>-23994.35</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="Q12" s="3" t="n">
         <v>62</v>
       </c>
-      <c r="R12" t="n">
+      <c r="R12" s="3" t="n">
         <v>26.5</v>
       </c>
-      <c r="S12" t="n">
+      <c r="S12" s="3" t="n">
         <v>68.40000000000001</v>
       </c>
-      <c r="T12" t="n">
+      <c r="T12" s="3" t="n">
         <v>31503.37</v>
       </c>
-      <c r="U12" t="n">
+      <c r="U12" s="3" t="n">
         <v>-83391.92999999999</v>
       </c>
-      <c r="V12" t="n">
+      <c r="V12" s="3" t="n">
         <v>-91.5</v>
       </c>
-      <c r="W12" t="n">
+      <c r="W12" s="3" t="n">
         <v>175.2</v>
       </c>
-      <c r="X12" t="n">
+      <c r="X12" s="3" t="n">
         <v>-39110.26</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>CMP-08</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Cooking Oil 2L 1+1 Free App Coupon</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Multi-Buy BOGO</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Pantry Staples</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="3" t="n">
         <v>58000</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Margin Destroyer (Cherry-Picked &amp; Stockpiled)</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="3" t="n">
         <v>13557</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="3" t="n">
         <v>16.48592240171129</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="3" t="n">
         <v>3.354243564210371</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="3" t="n">
         <v>19.84016596592166</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="3" t="n">
         <v>11.59722504978978</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" s="3" t="n">
         <v>268973.13</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N13" s="3" t="n">
         <v>111749.55</v>
       </c>
-      <c r="O13" t="n">
+      <c r="O13" s="3" t="n">
         <v>157223.58</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P13" s="3" t="n">
         <v>-45851.49</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q13" s="3" t="n">
         <v>62</v>
       </c>
-      <c r="R13" t="n">
+      <c r="R13" s="3" t="n">
         <v>26.5</v>
       </c>
-      <c r="S13" t="n">
+      <c r="S13" s="3" t="n">
         <v>68.40000000000001</v>
       </c>
-      <c r="T13" t="n">
+      <c r="T13" s="3" t="n">
         <v>30931.91</v>
       </c>
-      <c r="U13" t="n">
+      <c r="U13" s="3" t="n">
         <v>-104171.23</v>
       </c>
-      <c r="V13" t="n">
+      <c r="V13" s="3" t="n">
         <v>-93.2</v>
       </c>
-      <c r="W13" t="n">
+      <c r="W13" s="3" t="n">
         <v>192.7</v>
       </c>
-      <c r="X13" t="n">
+      <c r="X13" s="3" t="n">
         <v>-53749.55</v>
       </c>
     </row>
@@ -1789,238 +1868,826 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="39" customWidth="1" min="15" max="15"/>
+    <col width="48" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>customer_archetype</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Total_Transactions</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Unique_Customers</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Avg_Net_Basket_EUR</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Avg_Items_Per_Basket</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Coupon_Usage_Rate_Pct</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Total_Net_Sales_EUR</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Total_Discount_Claimed_EUR</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Total_Net_Margin_EUR</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Recommended_CRM_Action</t>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>campaign_id</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>campaign_name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>mechanic_type</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Treatment_Sample_N</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Control_Holdout_N</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Control_Mean_Basket_EUR</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Treatment_Mean_Basket_EUR</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Observed_Basket_Diff_EUR</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Causal_DiD_Net_Uplift_EUR</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>CI_95_Lower_EUR</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>CI_95_Upper_EUR</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Welch_t_Statistic</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>p_Value</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Statistical_Power_Pct</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Causal_Margin_Impact_Per_Basket_EUR</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Board_Experiment_Decision</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>At-Risk / Slipping</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>42710</v>
-      </c>
-      <c r="C2" t="n">
-        <v>6032</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F2" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="G2" t="n">
-        <v>961153.73</v>
-      </c>
-      <c r="H2" t="n">
-        <v>42059.77</v>
-      </c>
-      <c r="I2" t="n">
-        <v>203726.93</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Automated Win-Back: Trigger €4 off €25 push notification after 18 days of scan inactivity.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>CMP-05</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Spend €40 Get €5 Off Family Stock-Up</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Basket Threshold (€40+)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>13735</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>6180</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>45.95</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>21.15</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>26.31</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>193.97</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Core Weekly Loyal</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>120934</v>
-      </c>
-      <c r="C3" t="n">
-        <v>17043</v>
-      </c>
-      <c r="D3" t="n">
-        <v>31.88</v>
-      </c>
-      <c r="E3" t="n">
-        <v>11</v>
-      </c>
-      <c r="F3" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>3855639.41</v>
-      </c>
-      <c r="H3" t="n">
-        <v>179776.22</v>
-      </c>
-      <c r="I3" t="n">
-        <v>808898.42</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Basket Stretch: Target with 'Spend €35 Get €3.50 Off' threshold coupons to lift basket from €29 to €36+.</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>CMP-02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Spend €30 Get €3 Off Weekend Basket</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Basket Threshold (€30+)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>13981</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>6291</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>47.93</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>23.13</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>26.03</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>25.77</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>26.29</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>195.55</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Promo-Driven Cherry Picker</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>77141</v>
-      </c>
-      <c r="C4" t="n">
-        <v>10899</v>
-      </c>
-      <c r="D4" t="n">
-        <v>22.04</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" t="n">
-        <v>78.09999999999999</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1700266.6</v>
-      </c>
-      <c r="H4" t="n">
-        <v>212363.47</v>
-      </c>
-      <c r="I4" t="n">
-        <v>256229.67</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Curb Cherry-Picking: Replace standalone deep item discounts with minimum €20 basket spend unlocks.</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CMP-07</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Digital Scratch Card €1.50 Instant Reward</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Gamified Scratch Card</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>13629</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>6133</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>16.66</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>16.92</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>123.58</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Single-Category Shopper</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>50333</v>
-      </c>
-      <c r="C5" t="n">
-        <v>7081</v>
-      </c>
-      <c r="D5" t="n">
-        <v>18.96</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>954563.72</v>
-      </c>
-      <c r="H5" t="n">
-        <v>62813.12</v>
-      </c>
-      <c r="I5" t="n">
-        <v>186443.18</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Cross-Category Halo: Trigger personalized bundled coupons pairing Bakery/Fruit with Dairy &amp; Meat.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CMP-12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Inactive 21-Day Win-Back €4 Off €25</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Win-Back Targeted</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>13641</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>6138</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>34.08</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>16.57</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>16.31</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>16.83</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>122.96</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>VIP Full-Basket Family</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>62519</v>
-      </c>
-      <c r="C6" t="n">
-        <v>8899</v>
-      </c>
-      <c r="D6" t="n">
-        <v>45.97</v>
-      </c>
-      <c r="E6" t="n">
-        <v>16</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CMP-01</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Baltic Fresh Bakery -30% App Coupon</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Category % Discount</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>13723</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>6175</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>38.3</v>
       </c>
-      <c r="G6" t="n">
-        <v>2874092.14</v>
-      </c>
-      <c r="H6" t="n">
-        <v>84790.98</v>
-      </c>
-      <c r="I6" t="n">
-        <v>640136.71</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Protect Margin: Avoid deep % discounts; reward with experiential perks, partner vouchers &amp; early access.</t>
+      <c r="H6" s="3" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>14.95</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>14.69</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>15.21</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>111.27</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>CMP-06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Bananas &amp; Berries -25% App Deal</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Category % Discount</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>13692</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>6161</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>38.47</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>14.86</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>110.48</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>CMP-09</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Baltic Grill &amp; Fresh Meat -20% Weekend</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Category % Discount</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>13681</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>6156</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>38.62</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>13.82</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>15.01</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>109.62</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CMP-03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Private Label Dairy &amp; Cheese -20%</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Category % Discount</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>13701</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>6165</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>35.74</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>11.36</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>82.55</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>CMP-10</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Organic &amp; BIO Range -25% Green Week</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Category % Discount</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>13944</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>6274</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>35.25</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>83.05</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>SCALE UP (Stat. Significant Positive Lift)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>CMP-04</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Imported Coffee Beans XXL -35% Promo</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Deep Item Discount</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>13379</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>6020</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>14.04</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>-10.76</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>-11.36</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>-11.63</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>-11.09</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>-83.48999999999999</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>-5.21</v>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>TERMINATE STANDALONE (Stat. Significant Margin Destruction)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>CMP-11</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Household Detergent XXL -40% Coupon</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Deep Item Discount</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>13806</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>6212</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>13.24</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>-11.56</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>-11.36</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>-11.62</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>-11.1</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>-84.81</v>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>-6.04</v>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>TERMINATE STANDALONE (Stat. Significant Margin Destruction)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>CMP-08</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Cooking Oil 2L 1+1 Free App Coupon</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Multi-Buy BOGO</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>13557</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>6100</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>-13.2</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>-11.36</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>-11.62</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>-11.1</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>-84.04000000000001</v>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 0.0001</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>-7.68</v>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>TERMINATE STANDALONE (Stat. Significant Margin Destruction)</t>
         </is>
       </c>
     </row>
@@ -2035,129 +2702,251 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Stage_Order</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Funnel_Stage</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Users_Count</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Conversion_From_Prev_Pct</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Overall_Penetration_Pct</t>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>customer_archetype</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Total_Transactions</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Unique_Customers</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Net_Basket_EUR</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Items_Per_Basket</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Coupon_Usage_Rate_Pct</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Total_Net_Sales_EUR</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Total_Discount_Claimed_EUR</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Total_Net_Margin_EUR</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Recommended_CRM_Action</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1. App Downloaded &amp; Registered</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E2" t="n">
-        <v>100</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>At-Risk / Slipping</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>42710</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>6032</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>961153.73</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>42059.77</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>203726.93</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Automated Win-Back: Trigger €4 off €25 push notification after 18 days of scan inactivity.</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2. First Digital Card Scan at POS</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>43600</v>
-      </c>
-      <c r="D3" t="n">
-        <v>87.2</v>
-      </c>
-      <c r="E3" t="n">
-        <v>87.2</v>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Core Weekly Loyal</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>120934</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>17043</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>31.88</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>3855639.41</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>179776.22</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>808898.42</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Basket Stretch: Target with 'Spend €35 Get €3.50 Off' threshold coupons to lift basket from €29 to €36+.</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Promo-Driven Cherry Picker</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>77141</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>10899</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>22.04</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>3. First Digital Coupon Activated &amp; Redeemed</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>36400</v>
-      </c>
-      <c r="D4" t="n">
-        <v>83.5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>72.8</v>
+      <c r="F4" s="3" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>1700266.6</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>212363.47</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>256229.67</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Curb Cherry-Picking: Replace standalone deep item discounts with minimum €20 basket spend unlocks.</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Single-Category Shopper</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>50333</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>7081</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>18.96</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>4. Repeat Active Shopper (3+ Visits / Month)</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>28900</v>
-      </c>
-      <c r="D5" t="n">
-        <v>79.40000000000001</v>
-      </c>
-      <c r="E5" t="n">
-        <v>57.8</v>
+      <c r="F5" s="3" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>954563.72</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>62813.12</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>186443.18</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Cross-Category Halo: Trigger personalized bundled coupons pairing Bakery/Fruit with Dairy &amp; Meat.</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>5. Habitual Loyal Advocate (Weekly Multi-Category)</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>21200</v>
-      </c>
-      <c r="D6" t="n">
-        <v>73.40000000000001</v>
-      </c>
-      <c r="E6" t="n">
-        <v>42.4</v>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>VIP Full-Basket Family</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>62519</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>8899</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>45.97</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>2874092.14</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>84790.98</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>640136.71</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Protect Margin: Avoid deep % discounts; reward with experiential perks, partner vouchers &amp; early access.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2171,204 +2960,1245 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Cohort_Month</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Acquired_Users</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>M0_Active_Pct</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>M1_Retained_Pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>M2_Retained_Pct</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>M3_Retained_Pct</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>M4_Retained_Pct</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>M5_Retained_Pct</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Monthly_Spend_EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-04 (Apr)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>9450</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>114.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-05 (May)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>8820</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="n">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-06 (Jun)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>8310</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="n">
+        <v>121.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07 (Jul)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7940</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="n">
+        <v>124.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08 (Aug)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>7860</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>84.09999999999999</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="n">
+        <v>126.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09 (Sep)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>7620</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="n">
+        <v>129.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>customer_archetype</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Active_Members</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Purchase_Frequency_Monthly</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Net_Basket_EUR</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Days_Since_Last_Scan</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Churn_Probability_30d_Pct</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Predicted_12M_CLV_EUR</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Predicted_12M_Net_Margin_EUR</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Annual_Revenue_At_Risk_EUR</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Predictive_Model_Trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>VIP Full-Basket Family</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>53.03</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>3480</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>782.5</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>200448</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Low Churn Risk: Enroll in Tier-1 Partner Perks &amp; Zero-Discount Brand Advocacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Core Weekly Loyal</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>17000</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>34.81</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>1695</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>368.4</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>409173</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Moderate Risk: Trigger €35 Basket Stretch Coupon if Scan Gap Exceeds 10 Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Single-Category Shopper</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>19.65</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>612</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>131.2</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>136231</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Medium Risk: Push Cross-Category Affinity Bundle (Bakery + Dairy -20%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Promo-Driven Cherry Picker</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>11000</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>584</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>285868</v>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Low Margin Retention: Restrict Standalone Deep Discounts; Enforce €20 Basket Floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>At-Risk / Slipping</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>23.43</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>392</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>160876</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL CHURN ALERT (&gt;65%): Automated 18-Day Push 'Spend €25 Get €4 Off' Win-Back</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Rule_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Anchor_Promo_Category</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Attached_Halo_Category</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Support_Pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Confidence_Pct</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Lift_Ratio</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Attached_Halo_Spend_EUR</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Avg_Attached_Margin_EUR</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Recommended_App_Bundle_Mechanic</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MBA-01</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Bakery (In-Store Oven)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Dairy, Butter &amp; Fresh Cheese</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Pair -25% Bakery App Coupon with 'Buy 2 Private Label Cheeses Get €1 Off'</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>MBA-02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Meat &amp; Poultry (Weekend Grill)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Fruit, Salad &amp; Craft Beverages</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Trigger Weekend Grill Cross-Coupon: Spend €15 on Meat + Produce for +€2.50 Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>MBA-03</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Bananas &amp; Berries</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Organic &amp; BIO Yogurt / Breakfast Cereals</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Target Single-Category Fruit Shoppers with BIO Breakfast Cross-Sell Push</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>MBA-04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Private Label Dairy &amp; Eggs</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Bakery &amp; Packaged Deli Meats</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Core Weekly Habit Anchor: Keep High Availability in Digital Scratch Card Rewards</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MBA-05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Organic &amp; BIO Range</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Premium Nuts, Dried Fruit &amp; Plant Milk</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>High-Margin VIP Segment Bundle: Spend €20 on BIO Range Get €3 Off</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>MBA-06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Imported Coffee Beans XXL (-35%)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>No Consistent Attachment (Standalone Cherry-Pick)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>LOW AFFINITY (Lift &lt; 1.0): Never Discount Standalone; Gate Behind €30 Total Basket</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>MBA-07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Cooking Oil 2L 1+1 Free</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>No Consistent Attachment (Stockpiled Staple)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>-3.45</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>NEGATIVE HALO (Lift 0.69): Eliminate BOGO; Replace with Multi-Category Spend Tier</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Mechanic_Category</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Current_H1_Budget_EUR</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Current_Historical_ROI_Pct</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Current_Net_Margin_Contribution_EUR</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Optimized_Q4_Budget_EUR</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Budget_Shift_EUR</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Projected_Q4_Net_Margin_EUR</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Optimization_Rationale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>1. High-Halo Fresh Anchors (Meat, Bakery, Fruit)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>145000</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>167620</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>235000</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>264800</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Expand +62% budget: Highest cross-category basket attachment (2.6x-3.1x lift) &amp; minimal post-dip</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2. Basket Stretch Thresholds (Spend €30/€40 Get €3/€5)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>143000</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>162.4</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>232230</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>215000</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>72000</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>341500</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Expand +50% budget: Forces basket size above €35+ floor; virtually eliminates cherry-picking (11.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>3. Private Label &amp; Organic Margin Builders</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>85000</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>118.2</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>100470</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>105000</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>122850</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Expand +24% budget: Builds long-term Private Label habit with higher gross margin baseline (28%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>4. Gamified Scratch Cards &amp; 18-Day Win-Back Triggers</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>81000</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>79785</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>70000</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>-11000</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>84200</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Focus strictly on 18-day inactive slipping shoppers; cap scratch card reward at €1.50 on €20+ spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>5. Standalone Deep Item Discounts (Coffee -35%, Oil BOGO, Detergent -40%)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>171000</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>-71.8</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>-122778</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>-171000</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PHASE OUT STANDALONE (-100%): Reallocate €171k away from cherry-picked stockpiling promos into €30+ thresholds</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Check_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Pipeline_Stage</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Issue_Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Records_Affected</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Pct_of_Total</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Remediation_Action</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>DQ-01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Raw POS Ingestion</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Total Raw POS Records Ingested</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>528390</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Loaded into staging table</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>DQ-02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Deduplication</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Duplicate Cashier / App Receipt Scans</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="3" t="n">
         <v>3420</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>0.65</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Deduplicated via ROW_NUMBER() OVER (PARTITION BY transaction_id, timestamp)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>DQ-03</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Refund Separation</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Negative Basket Values (Returns &amp; Refunds)</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="3" t="n">
         <v>2180</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>0.41</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Routed to separate fact_returns table to prevent basket size distortion</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>DQ-04</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Store ID Imputation</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Missing Terminal Store IDs</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="3" t="n">
         <v>1150</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>0.22</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Imputed via POS terminal IP &amp; country prefix mapping</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>DQ-05</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Coupon Reconciliation</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Activated App Coupon Not Applied at Checkout</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="3" t="n">
         <v>1640</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>0.31</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Flagged for CRM goodwill credit &amp; excluded from redeemed ROI</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>DQ-06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Gold Analytical Layer</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Clean Validated POS Sales Transactions</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="3" t="n">
         <v>520000</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="3" t="n">
         <v>98.41</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Promoted to Gold analytical fact table (99.98% accuracy)</t>
         </is>

</xml_diff>